<commit_message>
address ,case and design changes
</commit_message>
<xml_diff>
--- a/public/files/address_import.xlsx
+++ b/public/files/address_import.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -28,13 +28,22 @@
     <t xml:space="preserve">Pincode</t>
   </si>
   <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">624 High Road, Woodford Green, Greater London, IG8 0PU</t>
   </si>
   <si>
     <t xml:space="preserve"> IG8 0PU</t>
   </si>
   <si>
+    <t xml:space="preserve">address</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location</t>
   </si>
 </sst>
 </file>
@@ -72,13 +81,13 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -329,7 +338,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.81"/>
@@ -346,21 +355,30 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
+      <c r="A2" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
address,case and work detail page changes
</commit_message>
<xml_diff>
--- a/public/files/address_import.xlsx
+++ b/public/files/address_import.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -31,6 +31,9 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
+    <t xml:space="preserve">Short Name</t>
+  </si>
+  <si>
     <t xml:space="preserve">624 High Road, Woodford Green, Greater London, IG8 0PU</t>
   </si>
   <si>
@@ -38,6 +41,9 @@
   </si>
   <si>
     <t xml:space="preserve">address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Woodoffice green</t>
   </si>
   <si>
     <t xml:space="preserve">Test</t>
@@ -53,7 +59,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -75,12 +81,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -132,7 +132,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -142,10 +142,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -338,7 +334,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.81"/>
@@ -355,30 +351,39 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>4</v>
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
table filed name changes
</commit_message>
<xml_diff>
--- a/public/files/address_import.xlsx
+++ b/public/files/address_import.xlsx
@@ -22,16 +22,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
+    <t xml:space="preserve">Postcode Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postcode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postcode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Short Name</t>
   </si>
   <si>
     <t xml:space="preserve">624 High Road, Woodford Green, Greater London, IG8 0PU</t>
@@ -59,7 +59,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,10 +83,17 @@
       <family val="0"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Ubuntu"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Ubuntu"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -132,7 +139,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -142,6 +149,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -334,18 +353,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -354,37 +373,49 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" s="5" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" s="5" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>